<commit_message>
Add playbook detail page
</commit_message>
<xml_diff>
--- a/data/playbook-template.xlsx
+++ b/data/playbook-template.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="47">
   <si>
     <t>Fill in the playbook title and the label ID it belongs to. You can find label IDs in Admin → Labels. Only one row needed — do not add extra rows.</t>
   </si>
@@ -49,7 +49,10 @@
     <t>Product comes out watery or too thin</t>
   </si>
   <si>
-    <t>Evidence the assistant should collect during diagnosis. "type" must be one of the dropdown values. Set "required" to yes or no.</t>
+    <t>Evidence the assistant should collect during diagnosis. "type" must be one of the dropdown values. Set "required" to yes or no. "action_id" is optional and should match an ID in Admin -&gt; Actions.</t>
+  </si>
+  <si>
+    <t>action_id</t>
   </si>
   <si>
     <t>type</t>
@@ -64,6 +67,9 @@
     <t>Current hopper temperature reading</t>
   </si>
   <si>
+    <t>read_hopper_temp</t>
+  </si>
+  <si>
     <t>reading</t>
   </si>
   <si>
@@ -91,7 +97,7 @@
     <t>high</t>
   </si>
   <si>
-    <t>Diagnostic questions the assistant can ask the user. "when_to_ask" is optional — describe when this question is relevant.</t>
+    <t>Diagnostic questions the assistant can ask the user. "when_to_ask" and "action_id" are optional. If set, "action_id" must match an ID in Admin -&gt; Actions.</t>
   </si>
   <si>
     <t>question</t>
@@ -629,24 +635,26 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D100"/>
+  <dimension ref="A1:E100"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
     <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="3" max="3" width="25" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" ht="40" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -659,133 +667,139 @@
       <c r="D2" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E2" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="6" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="7" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="15" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="17" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="18" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="19" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="20" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="21" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="22" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="23" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="33" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="34" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="35" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="36" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="37" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="38" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="39" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="40" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="43" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="44" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="45" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="46" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="48" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="49" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="50" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="51" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="52" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="53" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="54" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="55" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="56" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="57" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="58" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="59" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="60" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="61" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="62" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="63" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="64" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="65" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="66" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="67" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="68" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="69" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="70" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="71" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="72" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="73" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="74" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="75" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="76" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="77" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="78" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="79" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="80" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="81" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="82" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="83" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="84" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="85" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="86" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="87" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="88" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="89" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="90" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="91" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="92" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="93" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="94" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="95" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="96" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="97" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="98" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="99" spans="3:4" x14ac:dyDescent="0.25"/>
-    <row r="100" spans="3:4" x14ac:dyDescent="0.25"/>
+        <v>17</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="6" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="7" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="9" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="10" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="17" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="18" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="19" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="20" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="21" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="22" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="29" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="31" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="32" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="33" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="34" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="35" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="36" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="37" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="39" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="40" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="41" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="42" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="43" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="44" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="45" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="46" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="47" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="48" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="49" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="50" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="51" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="52" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="53" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="54" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="55" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="56" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="57" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="58" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="59" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="60" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="61" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="62" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="63" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="64" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="65" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="66" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="67" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="68" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="69" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="70" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="71" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="72" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="73" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="74" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="75" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="76" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="77" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="78" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="79" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="80" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="81" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="82" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="83" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="84" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="85" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="86" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="87" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="88" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="89" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="90" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="91" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="92" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="93" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="94" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="95" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="96" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="97" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="98" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="99" spans="4:5" x14ac:dyDescent="0.25"/>
+    <row r="100" spans="4:5" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be one of: photo, reading, observation, action, confirmation" sqref="C10:C100">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be one of: photo, reading, observation, action, confirmation" sqref="D10:D100">
       <formula1>"photo,reading,observation,action,confirmation"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be one of: photo, reading, observation, action, confirmation" sqref="C3:C100">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be one of: photo, reading, observation, action, confirmation" sqref="D3:D100">
       <formula1>"photo,reading,observation,action,confirmation"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be one of: yes, no" sqref="D10:D100">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be one of: yes, no" sqref="E10:E100">
       <formula1>"yes,no"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be one of: yes, no" sqref="D3:D100">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be one of: yes, no" sqref="E3:E100">
       <formula1>"yes,no"</formula1>
     </dataValidation>
   </dataValidations>
@@ -807,7 +821,7 @@
   <sheetData>
     <row r="1" ht="40" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -818,27 +832,27 @@
         <v>6</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="3:3" x14ac:dyDescent="0.25"/>
@@ -957,54 +971,62 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
     <col min="2" max="2" width="50" customWidth="1"/>
     <col min="3" max="3" width="40" customWidth="1"/>
     <col min="4" max="4" width="30" customWidth="1"/>
+    <col min="5" max="5" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" ht="40" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1022,24 +1044,24 @@
   <sheetData>
     <row r="1" ht="40" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -1063,7 +1085,7 @@
   <sheetData>
     <row r="1" ht="40" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1074,27 +1096,27 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>